<commit_message>
docs: record M03 follow-up verification and status correction
- M03_CHECKPOINT: 2026-09-25 browser/DB evidence. All checks pass except
  the recovery link same-browser code exchange (blocked by link-preview
  consumption and the built-in mailer rate limit); resume steps recorded.
- CURRENT/HANDOFF: next action narrowed to the single remaining check.
- ROADMAP/PRD.xlsx: user-authorized status correction (M00-M02, M04-M06
  Done; M03, M07 In Progress).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -5608,7 +5608,7 @@
       </c>
       <c r="E6" s="8">
         <f>B7</f>
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="B7" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"Done")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="4" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B10" s="9">
         <f>IFERROR(B7/B6,0)</f>
-        <v>0.058823529411764705</v>
+        <v>0.35294117647058826</v>
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
@@ -8909,7 +8909,7 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -9144,7 +9144,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat(M08): PayMongo hosted checkout for merchandise payment
M08-P01 (approved): PayMongo replaces Stripe for the Philippines
deployment. The online payment charges the merchandise total after
discounts; shipping is paid to the courier on delivery.

- Pay action re-runs checkout_quote server-side, converts exact PHP
  strings to centavos, reconciles lines/subtotal/discount and refuses
  totals below PHP 1.00.
- Hosted Checkout Session via fetch (no new package); itemized lines,
  or one exact discounted line when a coupon applies.
- /checkout/success marks nothing paid; cancel returns to checkout.
  No DB writes, orders or stock changes (M09).
- PRD workbook, DECISIONS and derived docs updated; .env.example
  lists PAYMONGO_SECRET_KEY / PAYMONGO_WEBHOOK_SECRET.
- 7 new payment unit tests (35/35 pass); lint, typecheck, build pass.
  Browser verification pending a PayMongo test key.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Next.js (App Router) + TypeScript + Tailwind CSS + shadcn/ui + Supabase (Postgres/Auth/Storage) + Stripe + Zod + React Hook Form + Resend + Vercel + Sentry.</t>
+          <t>Next.js (App Router) + TypeScript + Tailwind CSS + shadcn/ui + Supabase (Postgres/Auth/Storage) + PayMongo + Zod + React Hook Form + Resend + Vercel + Sentry.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Stripe only for MVP.</t>
+          <t>PayMongo only for MVP (M08-P01).</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2141,7 +2141,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>NEXT_PUBLIC_STRIPE_PUBLISHABLE_KEY</t>
+          <t>NEXT_PUBLIC_STRIPE_PUBLISHABLE_KEY (removed)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -2151,24 +2151,24 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Stripe client initialization</t>
+          <t>Not used: PayMongo hosted checkout needs no public key (M08-P01).</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Safe for browser.</t>
+          <t>Do not configure.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>STRIPE_SECRET_KEY</t>
+          <t>PAYMONGO_SECRET_KEY</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Create Stripe server-side resources</t>
+          <t>Create PayMongo checkout sessions</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -2195,7 +2195,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>STRIPE_WEBHOOK_SECRET</t>
+          <t>PAYMONGO_WEBHOOK_SECRET</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Verify Stripe webhook signatures</t>
+          <t>Verify PayMongo webhook signatures</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Stripe webhook authority</t>
+          <t>PayMongo webhook authority</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -3390,7 +3390,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>No service-role, Stripe secret, webhook secret, or email API keys in client/browser/logs.</t>
+          <t>No service-role, PayMongo secret, webhook secret, or email API keys in client/browser/logs.</t>
         </is>
       </c>
     </row>
@@ -3750,14 +3750,42 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="12" t="n"/>
-      <c r="C7" s="12" t="n"/>
-      <c r="D7" s="12" t="n"/>
-      <c r="E7" s="12" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="12" t="n"/>
+    <row r="7" ht="165" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>M08-P01</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Replace Stripe with PayMongo hosted checkout (supersedes D-001's payment provider only). M08 charges the merchandise total after discounts; shipping is paid to the courier on delivery. M08 authorized while M03/M07 stay In Progress for one open M03 check.</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Deployment is in the Philippines. Stripe does not list PH availability and local methods (GCash, Maya, QR Ph) are uncertain. PayMongo is PH-native with hosted checkout and signed webhooks.</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>01_EXEC_SUMMARY; 02_SCOPE; 03_ARCHITECTURE; 04_ROUTES; 05_DATA_MODEL; 07_ROADMAP; US-005; 10_ENV_INTEGRATIONS; 12_AI_GUARDRAILS. No new package; PAYMONGO_SECRET_KEY/PAYMONGO_WEBHOOK_SECRET replace Stripe env. No schema change in M08.</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>User (explicit session replies)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -5629,7 +5657,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -5640,7 +5668,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5671,7 +5699,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -5880,7 +5908,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>One Next.js repo; Supabase and Stripe are managed dependencies.</t>
+          <t>One Next.js repo; Supabase and PayMongo are managed dependencies.</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6212,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>M07-P01 approved: PHP; tax included. Third-party shipping fee and final payable total remain pending confirmation. No carrier integration.</t>
+          <t>M07-P01 approved: PHP; tax included. M08-P01 (2026-09-25): online payment charges the merchandise total after discounts; the customer pays the third-party courier's shipping fee directly on delivery. No carrier integration.</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6229,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Stripe payment flow</t>
+          <t>PayMongo hosted checkout payment flow</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -7015,7 +7043,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>PayMongo</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -7245,7 +7273,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Server creates Stripe payment/checkout session with metadata</t>
+          <t>Server creates PayMongo checkout session with metadata</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -7263,7 +7291,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Customer completes payment with Stripe</t>
+          <t>Customer completes payment on PayMongo hosted checkout</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -7281,7 +7309,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Stripe webhook is received and signature verified</t>
+          <t>PayMongo webhook is received and signature verified</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -7915,12 +7943,12 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>/api/stripe/webhook</t>
+          <t>/api/paymongo/webhook</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Stripe only</t>
+          <t>PayMongo only</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -7930,7 +7958,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Receive Stripe webhook</t>
+          <t>Receive PayMongo webhook</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -8288,7 +8316,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>id, user_id?, email, status, payment_status, subtotal, discount_total, shipping_total, tax_total, grand_total, currency, stripe refs, created_at</t>
+          <t>id, user_id?, email, status, payment_status, subtotal, discount_total, shipping_total, tax_total, grand_total, currency, payment provider refs (PayMongo; column rename proposed in M09), created_at</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -8379,7 +8407,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Stripe events</t>
+          <t>PayMongo events</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -9270,7 +9298,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Stripe payment</t>
+          <t>PayMongo payment</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -9285,12 +9313,12 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Stripe session/payment integration and safe metadata</t>
+          <t>PayMongo hosted checkout session and safe metadata; merchandise-only charge (shipping paid to courier on delivery)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(M09): record functional verification and In Progress status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -5657,7 +5657,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(M10): record functional verification and In Progress status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -5657,7 +5657,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -9407,7 +9407,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(M11): record functional verification and In Progress status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -5657,7 +5657,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(M12): record functional verification and In Progress status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -5657,7 +5657,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -9501,7 +9501,7 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(M13): record functional verification; PRD decision log M09-M13 and EMAIL_FROM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -35,7 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'07_ROADMAP'!$A$3:$I$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'08_USER_STORIES'!$A$3:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'09_COMPONENTS'!$A$3:$D$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'10_ENV_INTEGRATIONS'!$A$3:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'10_ENV_INTEGRATIONS'!$A$3:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'11_TEST_MATRIX'!$A$3:$F$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'12_AI_GUARDRAILS'!$A$3:$C$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'14_DECISION_LOG'!$A$3:$G$200</definedName>
@@ -2002,7 +2002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2327,8 +2327,35 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL_FROM</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Server only</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Sender for order confirmation email (M13-P01)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Testing: onboarding@resend.dev (delivers only to the Resend account owner). Verified own domain required before launch.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:E13"/>
+  <autoFilter ref="A3:E14"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -3787,41 +3814,153 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="12" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="12" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="12" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="12" t="n"/>
+    <row r="8" ht="165" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>M09-P01</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Verified PayMongo webhook creates exactly one paid order: provider-neutral payment_session_id/payment_id, immutable shipping_address snapshot, paid/unfulfilled/needs_review statuses; short stock or an over-limit coupon is recorded as needs_review without deducting stock; shipping_total 0 = paid to courier, tax_total 0 = included.</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Orders had no address fields and Stripe-named columns; paid customers must never lose an order to a race.</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>05_DATA_MODEL orders; US-006; T-001/T-004/T-005/T-006. Migration 20260928054657 (record_paid_checkout, service_role only).</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>User (explicit session replies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="165" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>M11-P01</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Admin catalog: archive over delete; product images JPEG/PNG/WebP up to 4 MB, checked by content and by the bucket; admin-only storage policies; stock set with an optimistic check (no log table).</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Storage had no upload policy or limits; concurrent stock edits must not overwrite sales.</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>02_SCOPE r19–r22; US-008/US-009; T-010/T-016. Migration 20260928073926.</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>User (explicit session replies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="165" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>M12-P01</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Fulfillment statuses Under review / To ship / Shipped / Delivered / Cancelled with fixed steps; courier and tracking number when shipping; order_status_history audit (admin read); one admin-only status function that cannot change payment state or amounts.</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>PRD requires allowed fulfillment statuses, protected payment status and auditable updates; orders had no update path.</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>02_SCOPE r21; US-010; 06_RLS_AUTH r13. Migrations 20260928081020 and 20260928081056.</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>User (explicit session replies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="165" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>M13-P01</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>One order confirmation per paid order via the Resend API: confirmation_email_sent_at plus Resend Idempotency-Key = order id; on failure the order is untouched, the error is logged and the webhook returns 500 so PayMongo retries the email. New EMAIL_FROM variable; testing uses onboarding@resend.dev.</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>PRD requires once per paid order, no duplicates on replayed webhooks, and failures logged without corrupting the order.</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>M13 roadmap; T-004; 10_ENV_INTEGRATIONS RESEND_API_KEY + EMAIL_FROM. Migration 20260928082612.</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>User (explicit session replies)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -5657,7 +5796,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -5668,7 +5807,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5699,7 +5838,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -9548,7 +9687,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore(M14): remove temporary monitoring test; record verification
Removes the admin test buttons and action. Docs and PRD: M14 In
Progress, decision log row 12, NEXT_PUBLIC_SENTRY_DSN env row, and the
Vercel function-log finding for M15.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -2276,12 +2276,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>SENTRY_DSN / related</t>
+          <t>NEXT_PUBLIC_SENTRY_DSN</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Scrub PII/secrets.</t>
+          <t>Scrub PII/secrets. A DSN is safe in the browser; lib/monitoring/scrub.ts masks emails and keys and drops request/user data (M14-P01). Monitoring is off when unset.</t>
         </is>
       </c>
     </row>
@@ -3962,14 +3962,42 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="12" t="n"/>
+    <row r="12" ht="165" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>M14-P01</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Sentry (@sentry/nextjs) errors only: no tracing, replay or default PII; every event scrubbed (request cookies/headers/bodies/query and user fields dropped; emails and PayMongo/Resend/Supabase keys, webhook secrets, JWTs and provider ids masked). Vercel Web Analytics (cookieless). onRequestError awaits a Sentry flush.</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>PRD requires visible production errors with no secret or PII leakage. On Vercel, server errors were captured but lost unless the flush was awaited.</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>M14 roadmap; 12_AI_GUARDRAILS r24; 10_ENV NEXT_PUBLIC_SENTRY_DSN. Packages @sentry/nextjs 11.0.0 and @vercel/analytics 2.0.1.</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>User (explicit session replies)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -5796,7 +5824,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -5807,7 +5835,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5838,7 +5866,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -9734,7 +9762,7 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(M15): record security review, fixes (M15-P01 proposed) and exact resume point
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -3999,14 +3999,42 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="12" t="n"/>
+    <row r="13" ht="165" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>M15-P01</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Security fixes found in the M15 review: Referrer-Policy changed from no-referrer to same-origin (no-referrer made browsers send Origin: null on non-JS form posts, so Next.js aborted Server Actions as CSRF: the old M03 login HTTP 500); X-Frame-Options DENY, CSP frame-ancestors none and X-Content-Type-Options nosniff on every response.</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Review evidence: RLS/grants/functions clean; T-007 to T-016 pass; no server secrets in browser bundles; webhook forgery/stale/replay/mode rejected. The two fixes were implemented within M15 scope and need explicit user confirmation.</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>12_AI_GUARDRAILS r13–r17, r24; 11_TEST_MATRIX T-007–T-016; proxy.ts, next.config.ts. A full Content-Security-Policy is recommended, not implemented.</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Claude (awaiting user confirmation)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -5824,7 +5852,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -5835,7 +5863,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5866,7 +5894,7 @@
       </c>
       <c r="E9" s="8">
         <f>B6-B7-B8-B9</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -9809,7 +9837,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs(M15): record M15-P01 as Approved
User approved M15-P01 (Referrer-Policy same-origin; anti-framing and
nosniff headers) on 2026-09-30. PRD 14_DECISION_LOG row 13: F13
Approved, G13 user, D13 evidence text; only sheet16.xml changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -4017,7 +4017,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Review evidence: RLS/grants/functions clean; T-007 to T-016 pass; no server secrets in browser bundles; webhook forgery/stale/replay/mode rejected. The two fixes were implemented within M15 scope and need explicit user confirmation.</t>
+          <t>Review evidence: RLS/grants/functions clean; T-007 to T-016 pass; no server secrets in browser bundles; webhook forgery/stale/replay/mode rejected. The two fixes were implemented within M15 scope and approved by the user on 2026-09-30.</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -4027,12 +4027,12 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Claude (awaiting user confirmation)</t>
+          <t>User (explicit session reply, 2026-09-30)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(M16): M16-P01 soft launch; stop webhook retries on permanent email refusals
Without a sending domain, Resend refuses customer addresses (403), which
made the webhook return 500 forever and PayMongo retry every real order.
A 4xx other than 408/409/429 is now logged as email_rejected and
acknowledged with 200; transient failures still return 500. Record
M16-P01 (Approved) in DECISIONS.md and PRD 14_DECISION_LOG row 14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -4036,14 +4036,42 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="12" t="n"/>
+    <row r="14" ht="165" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>M16-P01</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Soft launch on https://atleteka.vercel.app without a custom domain, guest checkout only. A permanent Resend refusal (HTTP 4xx except 408, 409, 429) of the order confirmation is logged and the webhook returns 200, so PayMongo stops retrying; transient failures still return 500 and are retried. Supabase Site URL and redirect URL set to atleteka.vercel.app.</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>No domain yet: the Resend test sender only delivers to the account owner and the built-in Supabase mailer is rate limited, so customer emails cannot be delivered. Without this change every real order would make PayMongo retry the webhook indefinitely. Accounts are not offered to customers until a domain exists.</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Amends M13-P01 (retry until the email succeeds). lib/email/retry.ts, app/api/paymongo/webhook/route.ts, tests/email.test.mjs. Reversal: verify a domain in Resend, set EMAIL_FROM and Supabase custom SMTP.</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>User (explicit session reply, 2026-09-30)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>

</xml_diff>

<commit_message>
docs(prd): close M03 and M07 in PRD.xlsx after the password-reset check passed
User-approved 2026-10-05. Cell-level edit: 07_ROADMAP E7 and E11 set to
Done; 15_DASHBOARD cached values 8 Done / 8 In Progress / 47.06%. Only
xl/worksheets/sheet2.xml and sheet9.xml were replaced; all other parts
verified byte-identical. ROADMAP.md, CURRENT.md and M03_CHECKPOINT.md
updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PRD.xlsx
+++ b/docs/PRD.xlsx
@@ -5859,7 +5859,7 @@
       </c>
       <c r="E6" s="8">
         <f>B7</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="B7" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"Done")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="4" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="E7" s="8">
         <f>B8</f>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('07_ROADMAP'!E4:E100,"In Progress")</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="4" t="inlineStr">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="B10" s="9">
         <f>IFERROR(B7/B6,0)</f>
-        <v>0.35294117647058826</v>
+        <v>0.47058823529411764</v>
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
@@ -9301,7 +9301,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -9489,7 +9489,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">

</xml_diff>